<commit_message>
Lịch lớp học: xem trước lịch các lớp sắp tới để chủ động sắp xếp thời gian
- /lop-hoc có 2 chế độ xem Danh sách | Lịch (mọi người xem được): lưới tháng chấm màu theo lớp,
  lớp Dự kiến công khai sớm hiện đủ Bài + giờ + slot (nhãn "Sắp mở"), vạch đỏ ngày còn thiếu người,
  nhãn riêng Bạn dạy / Trùng lịch của bạn / Phù hợp với bạn + lọc "Phù hợp với tôi"
- RPC lich_lop_hoc (migration 20261026100000), không lộ nhãn nhóm; test 18 kiểm tra
- "Công khai sớm" mặc định bật (form + CSV); thông báo "Lớp sắp mở đăng ký"
- Lưới tháng dùng chung (LuoiThang) cho cả Lịch dạy của tôi; icon lịch của Admin thuần mở lịch lớp
- Cập nhật CLAUDE.md, kế hoạch, tài liệu hướng dẫn (ảnh 3.2, 3.2b, 5.2; dựng lại PDF + Word), file mẫu CSV

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mau tao lop.xlsx
+++ b/mau tao lop.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="83">
   <si>
     <t>Mỗi dòng trong sheet "Mẫu tạo lớp" là 1 Bài. Các cột của lớp chỉ cần điền ở dòng Bài đầu tiên của mỗi mã lớp — dòng sau để trống là tự lấy lại giá trị dòng trước.</t>
   </si>
@@ -114,60 +114,63 @@
     <t>công khai sớm</t>
   </si>
   <si>
-    <t>"có" hoặc "không" — cho GV/TG thấy lớp khi còn Dự kiến.</t>
+    <t>"có" hoặc "không" — để trống = "có": GV/TG thấy lớp trên Lịch lớp học khi còn Dự kiến.</t>
+  </si>
+  <si>
+    <t>có</t>
+  </si>
+  <si>
+    <t>tên bài</t>
+  </si>
+  <si>
+    <t>Nội dung của buổi học (Bài) đó.</t>
+  </si>
+  <si>
+    <t>Lý thuyết hồi sinh tim phổi</t>
+  </si>
+  <si>
+    <t>ngày</t>
+  </si>
+  <si>
+    <t>Định dạng dd/mm/yyyy.</t>
+  </si>
+  <si>
+    <t>15/03/2026</t>
+  </si>
+  <si>
+    <t>giờ bắt đầu / giờ kết thúc</t>
+  </si>
+  <si>
+    <t>Định dạng HH:mm (giờ Việt Nam).</t>
+  </si>
+  <si>
+    <t>08:00 / 11:00</t>
+  </si>
+  <si>
+    <t>số giảng viên / số trợ giảng</t>
+  </si>
+  <si>
+    <t>Số nguyên 0–20; tổng 2 cột phải ≥ 1.</t>
+  </si>
+  <si>
+    <t>1 / 3</t>
+  </si>
+  <si>
+    <t>giờ bắt đầu</t>
+  </si>
+  <si>
+    <t>giờ kết thúc</t>
+  </si>
+  <si>
+    <t>số giảng viên</t>
+  </si>
+  <si>
+    <t>số trợ giảng</t>
   </si>
   <si>
     <t>không</t>
   </si>
   <si>
-    <t>tên bài</t>
-  </si>
-  <si>
-    <t>Nội dung của buổi học (Bài) đó.</t>
-  </si>
-  <si>
-    <t>Lý thuyết hồi sinh tim phổi</t>
-  </si>
-  <si>
-    <t>ngày</t>
-  </si>
-  <si>
-    <t>Định dạng dd/mm/yyyy.</t>
-  </si>
-  <si>
-    <t>15/03/2026</t>
-  </si>
-  <si>
-    <t>giờ bắt đầu / giờ kết thúc</t>
-  </si>
-  <si>
-    <t>Định dạng HH:mm (giờ Việt Nam).</t>
-  </si>
-  <si>
-    <t>08:00 / 11:00</t>
-  </si>
-  <si>
-    <t>số giảng viên / số trợ giảng</t>
-  </si>
-  <si>
-    <t>Số nguyên 0–20; tổng 2 cột phải ≥ 1.</t>
-  </si>
-  <si>
-    <t>1 / 3</t>
-  </si>
-  <si>
-    <t>giờ bắt đầu</t>
-  </si>
-  <si>
-    <t>giờ kết thúc</t>
-  </si>
-  <si>
-    <t>số giảng viên</t>
-  </si>
-  <si>
-    <t>số trợ giảng</t>
-  </si>
-  <si>
     <t>08:00</t>
   </si>
   <si>
@@ -210,9 +213,6 @@
     <t>Giảng viên không là bác sĩ;Trợ giảng không là bác sĩ</t>
   </si>
   <si>
-    <t>có</t>
-  </si>
-  <si>
     <t>Buổi duy nhất</t>
   </si>
   <si>
@@ -237,19 +237,16 @@
     <t>Ban giám đốc</t>
   </si>
   <si>
-    <t>Demo GD10-full CC-Hiếm</t>
+    <t>Chứng chỉ hành nghề</t>
   </si>
   <si>
     <t>Giảng viên là bác sĩ</t>
   </si>
   <si>
-    <t>Chứng chỉ hành nghề</t>
+    <t>Chứng chỉ sư phạm Y học</t>
   </si>
   <si>
     <t>Giảng viên không là bác sĩ</t>
-  </si>
-  <si>
-    <t>Chứng chỉ sư phạm Y học</t>
   </si>
   <si>
     <t>SCC-LX</t>
@@ -973,7 +970,7 @@
         <v>25</v>
       </c>
       <c r="I2" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="J2" t="s">
         <v>37</v>
@@ -982,10 +979,10 @@
         <v>40</v>
       </c>
       <c r="L2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="M2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N2">
         <v>1</v>
@@ -1023,16 +1020,16 @@
         <v>25</v>
       </c>
       <c r="J3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K3" t="s">
         <v>40</v>
       </c>
       <c r="L3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N3">
         <v>1</v>
@@ -1070,16 +1067,16 @@
         <v>25</v>
       </c>
       <c r="J4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="M4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N4">
         <v>1</v>
@@ -1090,31 +1087,31 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H5" t="s">
         <v>25</v>
       </c>
       <c r="I5" t="s">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="J5" t="s">
         <v>66</v>
@@ -1123,7 +1120,7 @@
         <v>67</v>
       </c>
       <c r="L5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="M5" t="s">
         <v>68</v>
@@ -1144,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1186,35 +1183,35 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B4" t="s">
         <v>77</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" t="s">
         <v>79</v>
       </c>
-      <c r="B5" t="s">
-        <v>80</v>
-      </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" t="s">
         <v>81</v>
       </c>
-      <c r="B6" t="s">
-        <v>82</v>
-      </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1225,18 +1222,7 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>